<commit_message>
data: sync verified Bosch source archive and published exports
</commit_message>
<xml_diff>
--- a/docs/downloads/bosch-kompendium.xlsx
+++ b/docs/downloads/bosch-kompendium.xlsx
@@ -844,7 +844,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">
@@ -891,7 +891,7 @@
       <c r="L4" s="4" t="n"/>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N4" s="7" t="inlineStr">
@@ -991,7 +991,7 @@
       <c r="L6" s="4" t="n"/>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N6" s="7" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="C12" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" s="6">
         <f>IF(AND(ISNUMBER(D12),ISNUMBER(E12)),SUM(D12:E12),"")</f>
@@ -1303,7 +1303,7 @@
       <c r="L12" s="4" t="n"/>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr">
@@ -1324,7 +1324,7 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>1</v>
@@ -1340,17 +1340,17 @@
         <v>1</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" s="4" t="n"/>
       <c r="K13" s="4" t="n"/>
       <c r="L13" s="4" t="n"/>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>0</v>
@@ -1980,7 +1980,7 @@
       <c r="L25" s="4" t="n"/>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
@@ -2080,7 +2080,7 @@
       <c r="L27" s="4" t="n"/>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
@@ -2233,7 +2233,7 @@
       <c r="L30" s="4" t="n"/>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N30" s="7" t="inlineStr">
@@ -2604,7 +2604,7 @@
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N38" s="7" t="inlineStr">
@@ -2731,7 +2731,7 @@
         </is>
       </c>
       <c r="C40" s="5" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D40" s="5" t="n">
         <v>22</v>
@@ -2757,7 +2757,7 @@
       <c r="L40" s="4" t="n"/>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N40" s="7" t="inlineStr">
@@ -2804,7 +2804,7 @@
       <c r="L41" s="4" t="n"/>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N41" s="7" t="inlineStr">
@@ -2957,7 +2957,7 @@
       <c r="L44" s="4" t="n"/>
       <c r="M44" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N44" s="7" t="inlineStr">
@@ -3004,7 +3004,7 @@
       <c r="L45" s="4" t="n"/>
       <c r="M45" s="4" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N45" s="7" t="inlineStr">

</xml_diff>

<commit_message>
data: publish verified Bosch Excel and source gap reports
</commit_message>
<xml_diff>
--- a/docs/downloads/bosch-kompendium.xlsx
+++ b/docs/downloads/bosch-kompendium.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Informacje" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zawodnicy" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sezony" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mecze" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Występy" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bramki" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Braki danych" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Informacje" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Zawodnicy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sezony" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Mecze" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Występy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Bramki" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Braki danych" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Zawodnicy'!$A$1:$N$46</definedName>

</xml_diff>

<commit_message>
fix: reconcile rejected video links and publish observed goal cues
</commit_message>
<xml_diff>
--- a/docs/downloads/bosch-kompendium.xlsx
+++ b/docs/downloads/bosch-kompendium.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Informacje" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Zawodnicy" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sezony" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mecze" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Występy" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Bramki" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Braki danych" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Informacje" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zawodnicy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sezony" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mecze" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Występy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bramki" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Braki danych" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Zawodnicy'!$A$1:$N$46</definedName>

</xml_diff>

<commit_message>
Fix portable workbook caching and complete source-backed halves analysis
</commit_message>
<xml_diff>
--- a/docs/downloads/bosch-kompendium.xlsx
+++ b/docs/downloads/bosch-kompendium.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Informacje" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Zawodnicy" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sezony" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mecze" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Występy" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Bramki" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Braki danych" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Informacje" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zawodnicy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sezony" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mecze" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Występy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bramki" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Braki danych" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Zawodnicy'!$A$1:$N$46</definedName>
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Mecze'!$A$1:$J$114</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Występy'!$A$1:$K$989</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Bramki'!$A$1:$I$221</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Braki danych'!$A$1:$F$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Braki danych'!$A$1:$F$31</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -64822,7 +64822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -64886,9 +64886,9 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -64900,140 +64900,140 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>2203</t>
+          <t>7266</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Bayer Emilian</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
+          <t>Bazyluk Jakub</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>NIE</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>plp_sportspress_player_id</t>
+          <t>plp_official_match_page_linked_id</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>7266</t>
+          <t>8654</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Bazyluk Jakub</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
+          <t>Bączek Szymon</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>TAK</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>plp_official_match_page_linked_id</t>
+          <t>PLP</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>8654</t>
+          <t>10321</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Bączek Szymon</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
+          <t>Ciborowski Julian</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>NIE</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_official_match_page_linked_id</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>10321</t>
+          <t>11895</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Ciborowski Julian</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
+          <t>Czudzinowicz Jakub (GK)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>TAK</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>plp_official_match_page_linked_id</t>
+          <t>plp_sportspress_player_id</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>11895</t>
+          <t>13196</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Czudzinowicz Jakub (GK)</t>
+          <t>Damian Rogon</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -65046,26 +65046,26 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>plp_sportspress_player_id</t>
+          <t>PLP</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>13196</t>
+          <t>2204</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Damian Rogon</t>
+          <t>Dawid Daniluk</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -65078,9 +65078,9 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -65092,12 +65092,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2204</t>
+          <t>7269</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Dawid Daniluk</t>
+          <t>Dołżyk Michał</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -65110,9 +65110,9 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -65124,12 +65124,12 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>7269</t>
+          <t>13197</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Dołżyk Michał</t>
+          <t>Filip Szparło</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -65142,9 +65142,9 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -65156,17 +65156,17 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>13197</t>
+          <t>7271</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Filip Szparło</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
+          <t>Gorbacewicz Emil</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -65181,19 +65181,19 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_official_match_page_linked_id</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>7271</t>
+          <t>7270</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Gorbacewicz Emil</t>
+          <t>Gołąbeski Piotr</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -65220,44 +65220,44 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>7270</t>
+          <t>7223</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Gołąbeski Piotr</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
+          <t>Grabowski Jakub (GK)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>TAK</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>plp_official_match_page_linked_id</t>
+          <t>plp_sportspress_player_id</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>7223</t>
+          <t>12425</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Grabowski Jakub (GK)</t>
+          <t>Karolczuk Jakub</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -65270,26 +65270,26 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>plp_sportspress_player_id</t>
+          <t>PLP</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>9400</t>
+          <t>10836</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Hyżyk Szymon</t>
+          <t>Karpiński Hubert</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -65297,14 +65297,14 @@
           <t>NIE</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>NIE</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -65316,12 +65316,12 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>7275</t>
+          <t>13194</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Jurkowicz Mateusz</t>
+          <t>Karpowicz Kamil</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -65329,14 +65329,14 @@
           <t>NIE</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>NIE</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -65348,22 +65348,22 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>7272</t>
+          <t>7278</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Jurkowicz Rafał</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
+          <t>Kossakowski Maciej</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -65373,19 +65373,19 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_official_match_page_linked_id</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>8914</t>
+          <t>9267</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Kadłubowski Krzysztof</t>
+          <t>Kowalczuk Karol</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -65393,14 +65393,14 @@
           <t>NIE</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>NIE</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -65412,76 +65412,76 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>1594</t>
+          <t>8655</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Kakareko Kamil</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
+          <t>Kuźma Gabriel</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>NIE</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>plp_sportspress_player_id</t>
+          <t>plp_official_match_page_linked_id</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>12425</t>
+          <t>7282</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Karolczuk Jakub</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
+          <t>Markowski Damian</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>NIE</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_official_match_page_linked_id</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>7276</t>
+          <t>8656</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Karolczuk Patryk</t>
+          <t>Muczyński Karol</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -65489,14 +65489,14 @@
           <t>NIE</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>NIE</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -65508,12 +65508,12 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>10836</t>
+          <t>12286</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Karpiński Hubert</t>
+          <t>Pietruczuk Paweł</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -65526,26 +65526,26 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_sportspress_player_id</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>13194</t>
+          <t>12290</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Karpowicz Kamil</t>
+          <t>Płochocki Maciej</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -65558,26 +65558,26 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>plp_sportspress_player_id</t>
+          <t>PLP</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>7277</t>
+          <t>12285</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Klepacki Przemysław</t>
+          <t>Rollauer Patryk</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -65585,68 +65585,68 @@
           <t>NIE</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>NIE</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_sportspress_player_id</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>7278</t>
+          <t>10603</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Kossakowski Maciej</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
+          <t>Roszkowski Patryk</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>TAK</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>plp_official_match_page_linked_id</t>
+          <t>plp_sportspress_player_id</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>9267</t>
+          <t>7285</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Kowalczuk Karol</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
+          <t>Sołowiej Tomasz</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -65661,19 +65661,19 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_official_match_page_linked_id</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>8655</t>
+          <t>7286</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Kuźma Gabriel</t>
+          <t>Uściłowski Krzysztof</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
@@ -65686,9 +65686,9 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -65700,12 +65700,12 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>4577</t>
+          <t>13198</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Kuźma Piotr</t>
+          <t>Wojciuk Piotr</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -65713,14 +65713,14 @@
           <t>NIE</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>NIE</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -65732,44 +65732,44 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>7280</t>
+          <t>8916</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Malinowski Piotr</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
+          <t>Wądołowski Sebastian</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>NIE</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_official_match_page_linked_id</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>7282</t>
+          <t>10604</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Markowski Damian</t>
+          <t>Śmiłowski Michał</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
@@ -65782,9 +65782,9 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -65796,12 +65796,12 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>12287</t>
+          <t>13010</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Mironiuk Zbigniew</t>
+          <t>Żak Paweł (GK)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -65809,504 +65809,24 @@
           <t>NIE</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>TAK</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>NIE</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
           <t>PLP</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>1960</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Moskal Paweł</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>PLP</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>8656</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Muczyński Karol</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>PLP</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>7283</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Nowicki Patryk</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>PLP</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>12286</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Pietruczuk Paweł</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>plp_sportspress_player_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>12290</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Płochocki Maciej</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>PLP</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>12285</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Rollauer Patryk</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>plp_sportspress_player_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>10603</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>Roszkowski Patryk</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>plp_sportspress_player_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>7284</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Rutkowski Mateusz (GK)</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>PLP</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>7285</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Sołowiej Tomasz</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>plp_official_match_page_linked_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>7286</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>Uściłowski Krzysztof</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>plp_official_match_page_linked_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>1970</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Wnuszyński Karol</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>PLP</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>13198</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Wojciuk Piotr</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>PLP</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>8916</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>Wądołowski Sebastian</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>plp_official_match_page_linked_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>10604</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Śmiłowski Michał</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>plp_official_match_page_linked_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>13010</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Żak Paweł (GK)</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>PLP</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F46"/>
+  <autoFilter ref="A1:F31"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Recover archived PLP portraits and allocate proven Supercup statistics
</commit_message>
<xml_diff>
--- a/docs/downloads/bosch-kompendium.xlsx
+++ b/docs/downloads/bosch-kompendium.xlsx
@@ -65169,14 +65169,14 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -65201,9 +65201,9 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -65366,9 +65366,9 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -65649,14 +65649,14 @@
           <t>TAK</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Explain untagged career events and allocate verified Supercup records and goal cue
</commit_message>
<xml_diff>
--- a/docs/downloads/bosch-kompendium.xlsx
+++ b/docs/downloads/bosch-kompendium.xlsx
@@ -3113,7 +3113,7 @@
         </is>
       </c>
       <c r="C45" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D45" s="5" t="n">
         <v>0</v>
@@ -3135,7 +3135,7 @@
         <v>0</v>
       </c>
       <c r="J45" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K45" s="5" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Reconstruct Bosch-only PLP careers with explicit scope evidence
</commit_message>
<xml_diff>
--- a/docs/downloads/bosch-kompendium.xlsx
+++ b/docs/downloads/bosch-kompendium.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Mecze'!$A$1:$J$114</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Występy'!$A$1:$M$989</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Bramki'!$A$1:$I$221</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Braki danych'!$A$1:$F$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Braki danych'!$A$1:$F$29</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -651,12 +651,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Minimum PLP — Sołowiej Tomasz</t>
+          <t>Rekonstrukcja PLP — Sołowiej Tomasz</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>apps: ≥33, goals: ≥22, assists: ≥13, motm: ≥3, yellow: ≥1, red: ≥0. Pełna kariera niepotwierdzona; odczyt publicznych protokołów.</t>
+          <t>apps: 33, goals: 22, assists: 13, motm: 3, yellow: 1, red: 0. Kariera zrekonstruowana z publicznych protokołów PLP. Użytkownik potwierdził 2026-10-19, że zawodnik grał w PLP wyłącznie w Boschu. Liczby pochodzą z protokołów; zakres klubowy z tego potwierdzenia. Aktualny publiczny profil pozostaje niedostępny.</t>
         </is>
       </c>
     </row>
@@ -687,12 +687,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Minimum PLP — Gołąbeski Piotr</t>
+          <t>Rekonstrukcja PLP — Gołąbeski Piotr</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>apps: ≥13, goals: ≥1, assists: ≥1, motm: ≥1, yellow: ≥4, red: ≥1. Pełna kariera niepotwierdzona; odczyt publicznych protokołów.</t>
+          <t>apps: 13, goals: 1, assists: 1, motm: 1, yellow: 4, red: 1. Kariera zrekonstruowana z publicznych protokołów PLP. Użytkownik potwierdził 2026-10-19, że zawodnik grał w PLP wyłącznie w Boschu. Liczby pochodzą z protokołów; zakres klubowy z tego potwierdzenia. Aktualny publiczny profil pozostaje niedostępny.</t>
         </is>
       </c>
     </row>
@@ -723,12 +723,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Minimum PLP — Gorbacewicz Emil</t>
+          <t>Rekonstrukcja PLP — Gorbacewicz Emil</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>apps: ≥10, goals: ≥0, assists: ≥3, motm: ≥0, yellow: ≥2, red: ≥0. Pełna kariera niepotwierdzona; odczyt publicznych protokołów.</t>
+          <t>apps: 10, goals: 0, assists: 3, motm: 0, yellow: 2, red: 0. Kariera zrekonstruowana z publicznych protokołów PLP. Użytkownik potwierdził 2026-10-19, że zawodnik grał w PLP wyłącznie w Boschu. Liczby pochodzą z protokołów; zakres klubowy z tego potwierdzenia. Aktualny publiczny profil pozostaje niedostępny.</t>
         </is>
       </c>
     </row>
@@ -747,24 +747,24 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Minimum PLP — Markowski Damian</t>
+          <t>Rekonstrukcja PLP — Markowski Damian</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>apps: ≥6, goals: ≥2, assists: ≥1, motm: ≥0, yellow: ≥0, red: ≥0. Pełna kariera niepotwierdzona; odczyt publicznych protokołów.</t>
+          <t>apps: 6, goals: 2, assists: 1, motm: 0, yellow: 0, red: 0. Kariera zrekonstruowana z publicznych protokołów PLP. Użytkownik potwierdził 2026-10-19, że zawodnik grał w PLP wyłącznie w Boschu. Liczby pochodzą z protokołów; zakres klubowy z tego potwierdzenia. Aktualny publiczny profil pozostaje niedostępny.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Minimum PLP — Kossakowski Maciej</t>
+          <t>Rekonstrukcja PLP — Kossakowski Maciej</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>apps: ≥5, goals: ≥0, assists: ≥0, motm: ≥0, yellow: ≥0, red: ≥0. Pełna kariera niepotwierdzona; odczyt publicznych protokołów.</t>
+          <t>apps: 5, goals: 0, assists: 0, motm: 0, yellow: 0, red: 0. Kariera zrekonstruowana z publicznych protokołów PLP. Użytkownik potwierdził 2026-10-19, że zawodnik grał w PLP wyłącznie w Boschu. Liczby pochodzą z protokołów; zakres klubowy z tego potwierdzenia. Aktualny publiczny profil pozostaje niedostępny.</t>
         </is>
       </c>
     </row>
@@ -783,72 +783,72 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Minimum PLP — Ciborowski Julian</t>
+          <t>Rekonstrukcja PLP — Ciborowski Julian</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>apps: ≥4, goals: ≥0, assists: ≥1, motm: ≥0, yellow: ≥0, red: ≥0. Pełna kariera niepotwierdzona; odczyt publicznych protokołów.</t>
+          <t>apps: 4, goals: 0, assists: 1, motm: 0, yellow: 0, red: 0. Kariera zrekonstruowana z publicznych protokołów PLP. Użytkownik potwierdził 2026-10-19, że zawodnik grał w PLP wyłącznie w Boschu. Liczby pochodzą z protokołów; zakres klubowy z tego potwierdzenia. Aktualny publiczny profil pozostaje niedostępny.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Minimum PLP — Śmiłowski Michał</t>
+          <t>Rekonstrukcja PLP — Śmiłowski Michał</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>apps: ≥1, goals: ≥0, assists: ≥0, motm: ≥0, yellow: ≥0, red: ≥0. Pełna kariera niepotwierdzona; odczyt publicznych protokołów.</t>
+          <t>apps: 1, goals: 0, assists: 0, motm: 0, yellow: 0, red: 0. Kariera zrekonstruowana z publicznych protokołów PLP. Użytkownik potwierdził 2026-10-19, że zawodnik grał w PLP wyłącznie w Boschu. Liczby pochodzą z protokołów; zakres klubowy z tego potwierdzenia. Aktualny publiczny profil pozostaje niedostępny.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Minimum PLP — Bazyluk Jakub</t>
+          <t>Rekonstrukcja PLP — Bazyluk Jakub</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>apps: ≥1, goals: ≥0, assists: ≥0, motm: ≥0, yellow: ≥1, red: ≥0. Pełna kariera niepotwierdzona; odczyt publicznych protokołów.</t>
+          <t>apps: 1, goals: 0, assists: 0, motm: 0, yellow: 1, red: 0. Kariera zrekonstruowana z publicznych protokołów PLP. Użytkownik potwierdził 2026-10-19, że zawodnik grał w PLP wyłącznie w Boschu. Liczby pochodzą z protokołów; zakres klubowy z tego potwierdzenia. Aktualny publiczny profil pozostaje niedostępny.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Minimum PLP — Uściłowski Krzysztof</t>
+          <t>Rekonstrukcja PLP — Uściłowski Krzysztof</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>apps: ≥2, goals: ≥0, assists: ≥0, motm: ≥0, yellow: ≥0, red: ≥0. Pełna kariera niepotwierdzona; odczyt publicznych protokołów.</t>
+          <t>apps: 2, goals: 0, assists: 0, motm: 0, yellow: 0, red: 0. Kariera zrekonstruowana z publicznych protokołów PLP. Użytkownik potwierdził 2026-10-19, że zawodnik grał w PLP wyłącznie w Boschu. Liczby pochodzą z protokołów; zakres klubowy z tego potwierdzenia. Aktualny publiczny profil pozostaje niedostępny.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Minimum PLP — Kuźma Gabriel</t>
+          <t>Rekonstrukcja PLP — Kuźma Gabriel</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>apps: ≥3, goals: ≥0, assists: ≥0, motm: ≥0, yellow: ≥0, red: ≥0. Pełna kariera niepotwierdzona; odczyt publicznych protokołów.</t>
+          <t>apps: 3, goals: 0, assists: 0, motm: 0, yellow: 0, red: 0. Kariera zrekonstruowana z publicznych protokołów PLP. Użytkownik potwierdził 2026-10-19, że zawodnik grał w PLP wyłącznie w Boschu. Liczby pochodzą z protokołów; zakres klubowy z tego potwierdzenia. Aktualny publiczny profil pozostaje niedostępny.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Minimum PLP — Wądołowski Sebastian</t>
+          <t>Rekonstrukcja PLP — Wądołowski Sebastian</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>apps: ≥1, goals: ≥0, assists: ≥0, motm: ≥0, yellow: ≥0, red: ≥0. Pełna kariera niepotwierdzona; odczyt publicznych protokołów.</t>
+          <t>apps: 1, goals: 0, assists: 0, motm: 0, yellow: 0, red: 0. Kariera zrekonstruowana z publicznych protokołów PLP. Użytkownik potwierdził 2026-10-19, że zawodnik grał w PLP wyłącznie w Boschu. Liczby pochodzą z protokołów; zakres klubowy z tego potwierdzenia. Aktualny publiczny profil pozostaje niedostępny.</t>
         </is>
       </c>
     </row>
@@ -1116,12 +1116,18 @@
       <c r="I4" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="6" t="n"/>
-      <c r="K4" s="6" t="n"/>
-      <c r="L4" s="6" t="n"/>
+      <c r="J4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Rekonstrukcja z protokołów</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
@@ -1222,12 +1228,18 @@
       <c r="I6" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="6" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="6" t="n"/>
+      <c r="J6" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Rekonstrukcja z protokołów</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
@@ -1552,17 +1564,23 @@
       <c r="I12" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="6" t="n"/>
-      <c r="K12" s="6" t="n"/>
-      <c r="L12" s="6" t="n"/>
+      <c r="J12" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <v>3</v>
+      </c>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Rekonstrukcja z protokołów</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>https://podlaskaliga.pl/wydarzenie/fc-grubassy-vs-bosch-service-tech-car-2/</t>
+          <t>https://podlaskaliga.pl/wydarzenie/top-auto-vs-bosch-service-tech-car/</t>
         </is>
       </c>
       <c r="O12" s="7" t="n">
@@ -1602,17 +1620,23 @@
       <c r="I13" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="J13" s="6" t="n"/>
-      <c r="K13" s="6" t="n"/>
-      <c r="L13" s="6" t="n"/>
+      <c r="J13" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Rekonstrukcja z protokołów</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>https://podlaskaliga.pl/wydarzenie/bosch-service-tech-car-vs-osmar-2/</t>
+          <t>https://podlaskaliga.pl/wydarzenie/bosch-service-tech-car-vs-fc-progress-bialystok/</t>
         </is>
       </c>
       <c r="O13" s="7" t="n">
@@ -2268,17 +2292,23 @@
       <c r="I25" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J25" s="6" t="n"/>
-      <c r="K25" s="6" t="n"/>
-      <c r="L25" s="6" t="n"/>
+      <c r="J25" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="M25" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Rekonstrukcja z protokołów</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>https://podlaskaliga.pl/wydarzenie/poler-art-team-vs-bosch-service-tech-car/</t>
+          <t>https://podlaskaliga.pl/wydarzenie/top-auto-vs-bosch-service-tech-car/</t>
         </is>
       </c>
       <c r="O25" s="7" t="n">
@@ -2374,12 +2404,18 @@
       <c r="I27" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J27" s="6" t="n"/>
-      <c r="K27" s="6" t="n"/>
-      <c r="L27" s="6" t="n"/>
+      <c r="J27" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="M27" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Rekonstrukcja z protokołów</t>
         </is>
       </c>
       <c r="N27" s="9" t="inlineStr">
@@ -2536,12 +2572,18 @@
       <c r="I30" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J30" s="6" t="n"/>
-      <c r="K30" s="6" t="n"/>
-      <c r="L30" s="6" t="n"/>
+      <c r="J30" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="K30" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="L30" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="M30" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Rekonstrukcja z protokołów</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
@@ -3090,17 +3132,23 @@
       <c r="I40" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J40" s="6" t="n"/>
-      <c r="K40" s="6" t="n"/>
-      <c r="L40" s="6" t="n"/>
+      <c r="J40" s="7" t="n">
+        <v>33</v>
+      </c>
+      <c r="K40" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="L40" s="7" t="n">
+        <v>13</v>
+      </c>
       <c r="M40" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Rekonstrukcja z protokołów</t>
         </is>
       </c>
       <c r="N40" s="9" t="inlineStr">
         <is>
-          <t>https://podlaskaliga.pl/wydarzenie/fc-grubassy-vs-bosch-service-tech-car-2/</t>
+          <t>https://podlaskaliga.pl/wydarzenie/top-auto-vs-bosch-service-tech-car/</t>
         </is>
       </c>
       <c r="O40" s="7" t="n">
@@ -3140,12 +3188,18 @@
       <c r="I41" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="6" t="n"/>
-      <c r="K41" s="6" t="n"/>
-      <c r="L41" s="6" t="n"/>
+      <c r="J41" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="M41" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Rekonstrukcja z protokołów</t>
         </is>
       </c>
       <c r="N41" s="9" t="inlineStr">
@@ -3302,12 +3356,18 @@
       <c r="I44" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J44" s="6" t="n"/>
-      <c r="K44" s="6" t="n"/>
-      <c r="L44" s="6" t="n"/>
+      <c r="J44" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="M44" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Rekonstrukcja z protokołów</t>
         </is>
       </c>
       <c r="N44" s="9" t="inlineStr">
@@ -3408,12 +3468,18 @@
       <c r="I46" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J46" s="6" t="n"/>
-      <c r="K46" s="6" t="n"/>
-      <c r="L46" s="6" t="n"/>
+      <c r="J46" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K46" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="M46" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Rekonstrukcja z protokołów</t>
         </is>
       </c>
       <c r="N46" s="9" t="inlineStr">
@@ -71178,7 +71244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -71264,9 +71330,9 @@
           <t>Bazyluk Jakub</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
@@ -71328,9 +71394,9 @@
           <t>Ciborowski Julian</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>TAK</t>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -71512,76 +71578,76 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>7271</t>
+          <t>7223</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Gorbacewicz Emil</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
+          <t>Grabowski Jakub (GK)</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>TAK</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>NIE</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>plp_official_match_page_linked_id</t>
+          <t>plp_sportspress_player_id</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>7270</t>
+          <t>12425</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Gołąbeski Piotr</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
+          <t>Karolczuk Jakub</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>TAK</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>NIE</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>plp_official_match_page_linked_id</t>
+          <t>PLP</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>7223</t>
+          <t>10836</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Grabowski Jakub (GK)</t>
+          <t>Karpiński Hubert</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -71601,19 +71667,19 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>plp_sportspress_player_id</t>
+          <t>PLP</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>12425</t>
+          <t>13194</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Karolczuk Jakub</t>
+          <t>Karpowicz Kamil</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -71633,19 +71699,19 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_sportspress_player_id</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>10836</t>
+          <t>7278</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Karpiński Hubert</t>
+          <t>Kossakowski Maciej</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -71665,19 +71731,19 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_official_match_page_linked_id</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>13194</t>
+          <t>9267</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Karpowicz Kamil</t>
+          <t>Kowalczuk Karol</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -71697,24 +71763,24 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>plp_sportspress_player_id</t>
+          <t>PLP</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>7278</t>
+          <t>8655</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Kossakowski Maciej</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>TAK</t>
+          <t>Kuźma Gabriel</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>NIE</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
@@ -71736,12 +71802,12 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>9267</t>
+          <t>7282</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Kowalczuk Karol</t>
+          <t>Markowski Damian</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -71761,31 +71827,31 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_official_match_page_linked_id</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>8655</t>
+          <t>8656</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Kuźma Gabriel</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
+          <t>Muczyński Karol</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>TAK</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
           <t>NIE</t>
@@ -71793,31 +71859,31 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>plp_official_match_page_linked_id</t>
+          <t>PLP</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>7282</t>
+          <t>12286</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Markowski Damian</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
+          <t>Pietruczuk Paweł</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>TAK</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
           <t>NIE</t>
@@ -71825,19 +71891,19 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>plp_official_match_page_linked_id</t>
+          <t>plp_sportspress_player_id</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>8656</t>
+          <t>12290</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Muczyński Karol</t>
+          <t>Płochocki Maciej</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -71864,12 +71930,12 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>12286</t>
+          <t>12285</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Pietruczuk Paweł</t>
+          <t>Rollauer Patryk</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -71896,12 +71962,12 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>12290</t>
+          <t>10603</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Płochocki Maciej</t>
+          <t>Roszkowski Patryk</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -71921,19 +71987,19 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_sportspress_player_id</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>12285</t>
+          <t>7286</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Rollauer Patryk</t>
+          <t>Uściłowski Krzysztof</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -71953,19 +72019,19 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>plp_sportspress_player_id</t>
+          <t>plp_official_match_page_linked_id</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>10603</t>
+          <t>13198</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Roszkowski Patryk</t>
+          <t>Wojciuk Piotr</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -71985,29 +72051,29 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>plp_sportspress_player_id</t>
+          <t>PLP</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>7285</t>
+          <t>8916</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Sołowiej Tomasz</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
+          <t>Wądołowski Sebastian</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>TAK</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>NIE</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -72024,24 +72090,24 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>7286</t>
+          <t>12288</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Uściłowski Krzysztof</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
+          <t>Zalewski Piotr</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
         <is>
           <t>TAK</t>
         </is>
       </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
           <t>NIE</t>
@@ -72049,19 +72115,19 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>plp_official_match_page_linked_id</t>
+          <t>PLP</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>13198</t>
+          <t>10604</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Wojciuk Piotr</t>
+          <t>Śmiłowski Michał</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -72081,31 +72147,31 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>PLP</t>
+          <t>plp_official_match_page_linked_id</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>8916</t>
+          <t>13010</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Wądołowski Sebastian</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="inlineStr">
+          <t>Żak Paweł (GK)</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>NIE</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
         <is>
           <t>TAK</t>
         </is>
       </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
           <t>NIE</t>
@@ -72113,108 +72179,12 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>plp_official_match_page_linked_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>12288</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>Zalewski Piotr</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D30" s="10" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
           <t>PLP</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>10604</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>Śmiłowski Michał</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="D31" s="10" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>plp_official_match_page_linked_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>13010</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>Żak Paweł (GK)</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>TAK</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>NIE</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>PLP</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F32"/>
+  <autoFilter ref="A1:F29"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Clarify scouting labels, restore all rival leaders and verify Bosch totals
</commit_message>
<xml_diff>
--- a/docs/downloads/bosch-kompendium.xlsx
+++ b/docs/downloads/bosch-kompendium.xlsx
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M3" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N19" s="9" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="M23" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="M35" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M37" s="6" t="inlineStr">
         <is>
-          <t>Potwierdzone minimum</t>
+          <t>Zweryfikowane sezony</t>
         </is>
       </c>
       <c r="N37" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Include verified Bosch Supercups in every player balance
</commit_message>
<xml_diff>
--- a/docs/downloads/bosch-kompendium.xlsx
+++ b/docs/downloads/bosch-kompendium.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Informacje" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Zawodnicy" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sezony" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mecze" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Występy" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Bramki" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Braki danych" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Informacje" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zawodnicy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sezony" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mecze" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Występy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bramki" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Braki danych" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Zawodnicy'!$A$1:$O$47</definedName>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>3</v>
@@ -1170,7 +1170,7 @@
         <v>2</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>12</v>
@@ -1823,10 +1823,10 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>16</v>
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D18" s="7" t="n">
         <v>28</v>
@@ -2047,13 +2047,13 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F21" s="8">
         <f>IF(AND(ISNUMBER(D21),ISNUMBER(E21)),SUM(D21:E21),"")</f>
@@ -2215,13 +2215,13 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D24" s="7" t="n">
         <v>24</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F24" s="8">
         <f>IF(AND(ISNUMBER(D24),ISNUMBER(E24)),SUM(D24:E24),"")</f>
@@ -2439,7 +2439,7 @@
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D28" s="7" t="n">
         <v>5</v>
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D29" s="7" t="n">
         <v>12</v>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="C31" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>1</v>
@@ -2663,10 +2663,10 @@
         </is>
       </c>
       <c r="C32" s="7" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D32" s="7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>33</v>
@@ -2775,13 +2775,13 @@
         </is>
       </c>
       <c r="C34" s="7" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D34" s="7" t="n">
         <v>22</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F34" s="8">
         <f>IF(AND(ISNUMBER(D34),ISNUMBER(E34)),SUM(D34:E34),"")</f>
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="C39" s="7" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D39" s="7" t="n">
         <v>2</v>
@@ -3223,7 +3223,7 @@
         </is>
       </c>
       <c r="C42" s="7" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D42" s="7" t="n">
         <v>13</v>

</xml_diff>